<commit_message>
Defense-ready release: UI redesign, async search, fixes, docs
- Apple-style dashboard redesign; Magic UI animations (NumberTicker,
  BlurFade), frosted sidebar, motion tokens, project logo + favicon
- Manufacturer search moved to background tasks: instant start, status
  polling, cancel endpoint, F5/navigation resume via localStorage
- Admin: deleting a user with history no longer fails on FK (documents
  and tasks detached, notifications removed)
- Task 1: use_llm flag — LLM verification opt-in via UI checkbox
- Task 2: iOS-style stepper, polished primary sumup table
- Infra: backend/frontend Dockerfiles, nginx.conf, .dockerignore,
  Magic UI MCP config; absolute upload paths; port 5433 defaults
- Docs: examples README, MacBook 8GB demo guide, thesis diagrams and
  screenshots
- Tests: 272 backend + 35 frontend green

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/Task2/synthetic/contract_registry_synthetic.xlsx
+++ b/examples/Task2/synthetic/contract_registry_synthetic.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Export" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM13"/>
+  <dimension ref="A1:BM68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46037</v>
+        <v>46028</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1000000</v>
+        <v>1050000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="AL4" s="1" t="n">
-        <v>46042</v>
+        <v>46038</v>
       </c>
       <c r="AM4" s="1" t="n">
         <v>46387</v>
@@ -585,11 +585,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DOG-AVIA-02</t>
+          <t>DOG-ARND-02</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46054</v>
+        <v>46029</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2500000</v>
+        <v>1300000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>р) закупки услуг в области воздушных перевозок и авиационных работ</t>
+          <t>л) закупки, предметом которых является аренда и (или) приобретение в собственность объектов недвижимого имущества</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -625,14 +625,14 @@
         </is>
       </c>
       <c r="AL5" s="1" t="n">
-        <v>46063</v>
+        <v>46039</v>
       </c>
       <c r="AM5" s="1" t="n">
         <v>46387</v>
       </c>
       <c r="BM5" t="inlineStr">
         <is>
-          <t>АО «Авиакомпания Лидер»</t>
+          <t>АО «Бизнес-Парк Северный»</t>
         </is>
       </c>
     </row>
@@ -644,11 +644,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DOG-INS-03</t>
+          <t>DOG-ARND-03</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46082</v>
+        <v>46030</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>850000</v>
+        <v>1550000</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>д) закупки финансовых услуг, включая страховые услуги</t>
+          <t>л) закупки, предметом которых является аренда и (или) приобретение в собственность объектов недвижимого имущества</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -684,14 +684,14 @@
         </is>
       </c>
       <c r="AL6" s="1" t="n">
-        <v>46086</v>
+        <v>46040</v>
       </c>
       <c r="AM6" s="1" t="n">
         <v>46387</v>
       </c>
       <c r="BM6" t="inlineStr">
         <is>
-          <t>АО СК «Надёжный Полис»</t>
+          <t>ООО «Городские Площади»</t>
         </is>
       </c>
     </row>
@@ -703,11 +703,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DOG-EDU-04</t>
+          <t>DOG-ARND-04</t>
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46073</v>
+        <v>46031</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>350000</v>
+        <v>1800000</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>ц) закупки услуг образовательных организаций</t>
+          <t>л) закупки, предметом которых является аренда и (или) приобретение в собственность объектов недвижимого имущества</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -743,14 +743,14 @@
         </is>
       </c>
       <c r="AL7" s="1" t="n">
-        <v>46082</v>
+        <v>46041</v>
       </c>
       <c r="AM7" s="1" t="n">
-        <v>46203</v>
+        <v>46387</v>
       </c>
       <c r="BM7" t="inlineStr">
         <is>
-          <t>АНО ДПО «Учебный Центр»</t>
+          <t>ЗАО «Офис Инвест»</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DOG-POST-05</t>
+          <t>DOG-ARND-05</t>
         </is>
       </c>
       <c r="C8" s="1" t="n">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>180000</v>
+        <v>2050000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>х) закупки услуг подвижной радиотелефонной связи</t>
+          <t>л) закупки, предметом которых является аренда и (или) приобретение в собственность объектов недвижимого имущества</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -802,14 +802,14 @@
         </is>
       </c>
       <c r="AL8" s="1" t="n">
-        <v>46037</v>
+        <v>46042</v>
       </c>
       <c r="AM8" s="1" t="n">
         <v>46387</v>
       </c>
       <c r="BM8" t="inlineStr">
         <is>
-          <t>ПАО «Связной Оператор»</t>
+          <t>ООО «АльфаРент»</t>
         </is>
       </c>
     </row>
@@ -821,11 +821,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DOG-SMSP-06</t>
+          <t>DOG-AVIA-01</t>
         </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46058</v>
+        <v>46055</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -833,26 +833,26 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>8000000</v>
+        <v>2100000</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>КИМ</t>
+          <t>ЕП</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Среднее</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Не является исключением</t>
+          <t>р) закупки услуг в области воздушных перевозок и авиационных работ</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -861,14 +861,14 @@
         </is>
       </c>
       <c r="AL9" s="1" t="n">
-        <v>46068</v>
+        <v>46060</v>
       </c>
       <c r="AM9" s="1" t="n">
         <v>46387</v>
       </c>
       <c r="BM9" t="inlineStr">
         <is>
-          <t>ООО «Средний Партнёр»</t>
+          <t>АО «Авиакомпания Лидер»</t>
         </is>
       </c>
     </row>
@@ -880,11 +880,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DOG-SMSP-07</t>
+          <t>DOG-AVIA-02</t>
         </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46091</v>
+        <v>46057</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -892,26 +892,26 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3200000</v>
+        <v>2700000</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>КИМ</t>
+          <t>ЕП</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Малое</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Не является исключением</t>
+          <t>р) закупки услуг в области воздушных перевозок и авиационных работ</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -920,14 +920,14 @@
         </is>
       </c>
       <c r="AL10" s="1" t="n">
-        <v>46096</v>
+        <v>46062</v>
       </c>
       <c r="AM10" s="1" t="n">
-        <v>46295</v>
+        <v>46387</v>
       </c>
       <c r="BM10" t="inlineStr">
         <is>
-          <t>ООО «Малый Поставщик»</t>
+          <t>ПАО «Аэрофлот»</t>
         </is>
       </c>
     </row>
@@ -939,11 +939,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DOG-MICRO-08</t>
+          <t>DOG-AVIA-03</t>
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46113</v>
+        <v>46059</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>450000</v>
+        <v>3300000</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Микро</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Не является исключением</t>
+          <t>р) закупки услуг в области воздушных перевозок и авиационных работ</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -979,14 +979,14 @@
         </is>
       </c>
       <c r="AL11" s="1" t="n">
-        <v>46122</v>
+        <v>46064</v>
       </c>
       <c r="AM11" s="1" t="n">
-        <v>46487</v>
+        <v>46387</v>
       </c>
       <c r="BM11" t="inlineStr">
         <is>
-          <t>ИП Иванов А.А.</t>
+          <t>ООО «Сибирские Авиалинии»</t>
         </is>
       </c>
     </row>
@@ -998,11 +998,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DOG-REG-09</t>
+          <t>DOG-AVIA-04</t>
         </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>46047</v>
+        <v>46061</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>750000</v>
+        <v>3900000</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Не является исключением</t>
+          <t>р) закупки услуг в области воздушных перевозок и авиационных работ</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1038,14 +1038,14 @@
         </is>
       </c>
       <c r="AL12" s="1" t="n">
-        <v>46054</v>
+        <v>46066</v>
       </c>
       <c r="AM12" s="1" t="n">
         <v>46387</v>
       </c>
       <c r="BM12" t="inlineStr">
         <is>
-          <t>ООО «Общий Поставщик»</t>
+          <t>АО «Уральские Перевозки»</t>
         </is>
       </c>
     </row>
@@ -1057,54 +1057,3299 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DOG-SMALL-10</t>
+          <t>DOG-INS-01</t>
         </is>
       </c>
       <c r="C13" s="1" t="n">
+        <v>46083</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>800000</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>д) закупки финансовых услуг, включая страховые услуги</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL13" s="1" t="n">
+        <v>46088</v>
+      </c>
+      <c r="AM13" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
+          <t>АО СК «Надёжный Полис»</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DOG-INS-02</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>46085</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>д) закупки финансовых услуг, включая страховые услуги</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL14" s="1" t="n">
+        <v>46090</v>
+      </c>
+      <c r="AM14" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM14" t="inlineStr">
+        <is>
+          <t>ООО СК «РосГарантия»</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DOG-INS-03</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>46087</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>д) закупки финансовых услуг, включая страховые услуги</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL15" s="1" t="n">
+        <v>46092</v>
+      </c>
+      <c r="AM15" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM15" t="inlineStr">
+        <is>
+          <t>АО «АльфаСтрахование»</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>DOG-INS-04</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>46089</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>д) закупки финансовых услуг, включая страховые услуги</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL16" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="AM16" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM16" t="inlineStr">
+        <is>
+          <t>ООО «Финансовый Партнёр»</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>DOG-EDU-01</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="n">
         <v>46065</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Поставка/услуги (синтетические данные)</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>280000</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>ц) закупки услуг образовательных организаций</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL17" s="1" t="n">
+        <v>46083</v>
+      </c>
+      <c r="AM17" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BM17" t="inlineStr">
+        <is>
+          <t>АНО ДПО «Учебный Центр»</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>DOG-EDU-02</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>46067</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>360000</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>ц) закупки услуг образовательных организаций</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL18" s="1" t="n">
+        <v>46084</v>
+      </c>
+      <c r="AM18" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BM18" t="inlineStr">
+        <is>
+          <t>ООО «Корпоративный Университет»</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DOG-EDU-03</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>46069</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>440000</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>ц) закупки услуг образовательных организаций</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL19" s="1" t="n">
+        <v>46085</v>
+      </c>
+      <c r="AM19" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BM19" t="inlineStr">
+        <is>
+          <t>ФГБОУ ВО «Технический Институт»</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>DOG-EDU-04</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="n">
+        <v>46071</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>520000</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>ц) закупки услуг образовательных организаций</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL20" s="1" t="n">
+        <v>46086</v>
+      </c>
+      <c r="AM20" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BM20" t="inlineStr">
+        <is>
+          <t>ООО «Бизнес-Школа Лидер»</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DOG-POST-01</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="n">
+        <v>46032</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>170000</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>х) закупки услуг подвижной радиотелефонной связи и услуг почтовой связи</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL21" s="1" t="n">
+        <v>46038</v>
+      </c>
+      <c r="AM21" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM21" t="inlineStr">
+        <is>
+          <t>ПАО «Связной Оператор»</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DOG-POST-02</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>220000</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>х) закупки услуг подвижной радиотелефонной связи и услуг почтовой связи</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL22" s="1" t="n">
+        <v>46039</v>
+      </c>
+      <c r="AM22" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM22" t="inlineStr">
+        <is>
+          <t>АО «МегаСвязь»</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DOG-POST-03</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>270000</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>х) закупки услуг подвижной радиотелефонной связи и услуг почтовой связи</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL23" s="1" t="n">
+        <v>46040</v>
+      </c>
+      <c r="AM23" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM23" t="inlineStr">
+        <is>
+          <t>ФГУП «Почта России»</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DOG-POST-04</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="n">
+        <v>46038</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>320000</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>х) закупки услуг подвижной радиотелефонной связи и услуг почтовой связи</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL24" s="1" t="n">
+        <v>46041</v>
+      </c>
+      <c r="AM24" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM24" t="inlineStr">
+        <is>
+          <t>ООО «Логистик Экспресс»</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MED-01</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>46056</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Среднее</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL25" s="1" t="n">
+        <v>46061</v>
+      </c>
+      <c r="AM25" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM25" t="inlineStr">
+        <is>
+          <t>ООО «Средний Партнёр»</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MED-02</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="n">
+        <v>46059</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Среднее</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL26" s="1" t="n">
+        <v>46064</v>
+      </c>
+      <c r="AM26" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM26" t="inlineStr">
+        <is>
+          <t>АО «Среднеотраслевые Решения»</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MED-03</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>46062</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>9500000</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Среднее</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL27" s="1" t="n">
+        <v>46067</v>
+      </c>
+      <c r="AM27" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM27" t="inlineStr">
+        <is>
+          <t>ООО «БетаПром»</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MED-04</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>11000000</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Среднее</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL28" s="1" t="n">
+        <v>46070</v>
+      </c>
+      <c r="AM28" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM28" t="inlineStr">
+        <is>
+          <t>АО «ГаммаЛогистик»</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MED-05</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="n">
+        <v>46068</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Среднее</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL29" s="1" t="n">
+        <v>46073</v>
+      </c>
+      <c r="AM29" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM29" t="inlineStr">
+        <is>
+          <t>ООО «Дельта-Консалтинг»</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-SMALL-01</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>46083</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL30" s="1" t="n">
+        <v>46088</v>
+      </c>
+      <c r="AM30" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="BM30" t="inlineStr">
+        <is>
+          <t>ООО «Малый Поставщик»</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-SMALL-02</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="n">
+        <v>46085</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL31" s="1" t="n">
+        <v>46090</v>
+      </c>
+      <c r="AM31" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="BM31" t="inlineStr">
+        <is>
+          <t>ООО «Эпсилон-Сервис»</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-SMALL-03</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="n">
+        <v>46087</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL32" s="1" t="n">
+        <v>46092</v>
+      </c>
+      <c r="AM32" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="BM32" t="inlineStr">
+        <is>
+          <t>ООО «Зета-Сетевик»</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-SMALL-04</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="n">
+        <v>46089</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>4400000</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL33" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="AM33" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="BM33" t="inlineStr">
+        <is>
+          <t>ООО «Эта-Решения»</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-SMALL-05</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="n">
+        <v>46091</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL34" s="1" t="n">
+        <v>46096</v>
+      </c>
+      <c r="AM34" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="BM34" t="inlineStr">
+        <is>
+          <t>ООО «Тета-Партнёр»</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-SMALL-06</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="n">
+        <v>46093</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>5600000</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>КИМ</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL35" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="AM35" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="BM35" t="inlineStr">
+        <is>
+          <t>ООО «Йота-Логистика»</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MICRO-01</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>450000</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL36" s="1" t="n">
+        <v>46119</v>
+      </c>
+      <c r="AM36" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="BM36" t="inlineStr">
+        <is>
+          <t>ИП Иванов А.А.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MICRO-02</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="n">
+        <v>46116</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>550000</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL37" s="1" t="n">
+        <v>46121</v>
+      </c>
+      <c r="AM37" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="BM37" t="inlineStr">
+        <is>
+          <t>ИП Смирнов В.К.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MICRO-03</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>650000</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL38" s="1" t="n">
+        <v>46123</v>
+      </c>
+      <c r="AM38" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="BM38" t="inlineStr">
+        <is>
+          <t>ООО «Каппа-Сервис»</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MICRO-04</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="n">
+        <v>46120</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>750000</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL39" s="1" t="n">
+        <v>46125</v>
+      </c>
+      <c r="AM39" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="BM39" t="inlineStr">
+        <is>
+          <t>ИП Кузнецов Д.С.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DOG-SMSP-MICRO-05</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="n">
+        <v>46122</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>850000</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL40" s="1" t="n">
+        <v>46127</v>
+      </c>
+      <c r="AM40" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="BM40" t="inlineStr">
+        <is>
+          <t>ООО «Лямбда-Микро»</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>DOG-WITH-SMALL-01</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="n">
+        <v>46115</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL41" s="1" t="n">
+        <v>46118</v>
+      </c>
+      <c r="AM41" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM41" t="inlineStr">
+        <is>
+          <t>ООО «Сигма-Технология»</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>DOG-WITH-SMALL-02</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL42" s="1" t="n">
+        <v>46121</v>
+      </c>
+      <c r="AM42" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM42" t="inlineStr">
+        <is>
+          <t>ООО «Тау-Сервис»</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>DOG-WITH-SMALL-03</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="n">
+        <v>46121</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL43" s="1" t="n">
+        <v>46124</v>
+      </c>
+      <c r="AM43" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM43" t="inlineStr">
+        <is>
+          <t>ООО «Ипсилон-Поставка»</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>DOG-WITH-SMALL-04</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="n">
+        <v>46124</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL44" s="1" t="n">
+        <v>46127</v>
+      </c>
+      <c r="AM44" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM44" t="inlineStr">
+        <is>
+          <t>ООО «Фи-Логистик»</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>DOG-WITH-SMALL-05</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>46127</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Малое</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL45" s="1" t="n">
+        <v>46130</v>
+      </c>
+      <c r="AM45" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM45" t="inlineStr">
+        <is>
+          <t>ООО «Хи-Решения»</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>DOG-WITH-MICRO-01</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>46144</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>330000</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL46" s="1" t="n">
+        <v>46147</v>
+      </c>
+      <c r="AM46" s="1" t="n">
+        <v>46356</v>
+      </c>
+      <c r="BM46" t="inlineStr">
+        <is>
+          <t>ИП Петров И.С.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>DOG-WITH-MICRO-02</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>410000</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL47" s="1" t="n">
+        <v>46149</v>
+      </c>
+      <c r="AM47" s="1" t="n">
+        <v>46356</v>
+      </c>
+      <c r="BM47" t="inlineStr">
+        <is>
+          <t>ИП Орлов М.В.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>DOG-WITH-MICRO-03</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="n">
+        <v>46148</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>490000</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL48" s="1" t="n">
+        <v>46151</v>
+      </c>
+      <c r="AM48" s="1" t="n">
+        <v>46356</v>
+      </c>
+      <c r="BM48" t="inlineStr">
+        <is>
+          <t>ООО «Пси-Микропоставка»</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>DOG-WITH-MICRO-04</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="n">
+        <v>46150</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>570000</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL49" s="1" t="n">
+        <v>46153</v>
+      </c>
+      <c r="AM49" s="1" t="n">
+        <v>46356</v>
+      </c>
+      <c r="BM49" t="inlineStr">
+        <is>
+          <t>ИП Соколов А.Н.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>DOG-WITH-MICRO-05</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="n">
+        <v>46152</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>650000</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL50" s="1" t="n">
+        <v>46155</v>
+      </c>
+      <c r="AM50" s="1" t="n">
+        <v>46356</v>
+      </c>
+      <c r="BM50" t="inlineStr">
+        <is>
+          <t>ИП Васильев Е.П.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>DOG-REG-01</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>750000</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL51" s="1" t="n">
+        <v>46055</v>
+      </c>
+      <c r="AM51" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM51" t="inlineStr">
+        <is>
+          <t>ООО «Общий Поставщик»</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>DOG-REG-02</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL52" s="1" t="n">
+        <v>46056</v>
+      </c>
+      <c r="AM52" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM52" t="inlineStr">
+        <is>
+          <t>АО «Стандарт-Сервис»</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>DOG-REG-03</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="n">
+        <v>46038</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1250000</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL53" s="1" t="n">
+        <v>46057</v>
+      </c>
+      <c r="AM53" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM53" t="inlineStr">
+        <is>
+          <t>ООО «РосТехОборудование»</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DOG-REG-04</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="n">
+        <v>46040</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL54" s="1" t="n">
+        <v>46058</v>
+      </c>
+      <c r="AM54" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM54" t="inlineStr">
+        <is>
+          <t>АО «ИндустриалПром»</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>DOG-REG-05</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="n">
+        <v>46042</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1750000</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL55" s="1" t="n">
+        <v>46059</v>
+      </c>
+      <c r="AM55" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM55" t="inlineStr">
+        <is>
+          <t>ООО «МегаСнаб»</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>DOG-REG-06</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL56" s="1" t="n">
+        <v>46060</v>
+      </c>
+      <c r="AM56" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM56" t="inlineStr">
+        <is>
+          <t>АО «Универсал-Логистик»</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>DOG-REG-07</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="n">
+        <v>46046</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>2250000</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL57" s="1" t="n">
+        <v>46061</v>
+      </c>
+      <c r="AM57" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM57" t="inlineStr">
+        <is>
+          <t>ООО «Промторг»</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>DOG-REG-08</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>46048</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL58" s="1" t="n">
+        <v>46062</v>
+      </c>
+      <c r="AM58" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM58" t="inlineStr">
+        <is>
+          <t>АО «БизнесЛидер»</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>DOG-SMALL-01</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="n">
+        <v>46061</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
         <v>45000</v>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>ЕП</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
         <is>
           <t>Не является исключением</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="AL13" s="1" t="n">
-        <v>46073</v>
-      </c>
-      <c r="AM13" s="1" t="n">
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL59" s="1" t="n">
+        <v>46066</v>
+      </c>
+      <c r="AM59" s="1" t="n">
         <v>46142</v>
       </c>
-      <c r="BM13" t="inlineStr">
+      <c r="BM59" t="inlineStr">
         <is>
           <t>ООО «Копеечный Сервис»</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>DOG-SMALL-02</t>
+        </is>
+      </c>
+      <c r="C60" s="1" t="n">
+        <v>46064</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL60" s="1" t="n">
+        <v>46069</v>
+      </c>
+      <c r="AM60" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="BM60" t="inlineStr">
+        <is>
+          <t>ИП Михайлов В.С.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>DOG-SMALL-03</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="n">
+        <v>46067</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL61" s="1" t="n">
+        <v>46072</v>
+      </c>
+      <c r="AM61" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="BM61" t="inlineStr">
+        <is>
+          <t>ООО «Малая Поставка»</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>DOG-SMALL-04</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>46070</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>90000</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL62" s="1" t="n">
+        <v>46075</v>
+      </c>
+      <c r="AM62" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="BM62" t="inlineStr">
+        <is>
+          <t>ИП Захаров А.Ю.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>DOG-CONT-01</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="n">
+        <v>45966</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>550000</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL63" s="1" t="n">
+        <v>45993</v>
+      </c>
+      <c r="AM63" s="1" t="n">
+        <v>46446</v>
+      </c>
+      <c r="BM63" t="inlineStr">
+        <is>
+          <t>ООО «Длящийся Сервис»</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>DOG-CONT-02</t>
+        </is>
+      </c>
+      <c r="C64" s="1" t="n">
+        <v>45971</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>700000</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL64" s="1" t="n">
+        <v>45994</v>
+      </c>
+      <c r="AM64" s="1" t="n">
+        <v>46474</v>
+      </c>
+      <c r="BM64" t="inlineStr">
+        <is>
+          <t>АО «Многолетние Поставки»</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>DOG-CONT-03</t>
+        </is>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>45976</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>850000</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Микро</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AL65" s="1" t="n">
+        <v>45995</v>
+      </c>
+      <c r="AM65" s="1" t="n">
+        <v>46505</v>
+      </c>
+      <c r="BM65" t="inlineStr">
+        <is>
+          <t>ООО «Долгосрочный Партнёр»</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>DOG-FRGN-01</t>
+        </is>
+      </c>
+      <c r="C66" s="1" t="n">
+        <v>46027</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AL66" s="1" t="n">
+        <v>46032</v>
+      </c>
+      <c r="AM66" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM66" t="inlineStr">
+        <is>
+          <t>ForeignCorp Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>DOG-FRGN-02</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="n">
+        <v>46032</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>700000</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AL67" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="AM67" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM67" t="inlineStr">
+        <is>
+          <t>EuroSupply GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>DOG-FRGN-03</t>
+        </is>
+      </c>
+      <c r="C68" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Поставка/услуги (синтетические данные)</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>900000</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>ЕП</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Не является исключением</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AL68" s="1" t="n">
+        <v>46042</v>
+      </c>
+      <c r="AM68" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="BM68" t="inlineStr">
+        <is>
+          <t>Asia Trading Co.</t>
         </is>
       </c>
     </row>

</xml_diff>